<commit_message>
Atualiza planilha de vagas pela sincronizacao Windows
</commit_message>
<xml_diff>
--- a/automacao_azure_devops/vagas.xlsx
+++ b/automacao_azure_devops/vagas.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\t.douglas.medeiros\Projeto Teste 1\automacao_azure_devops\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\t.douglas.medeiros\Desktop\dmma-dashboard-main\dmma-dashboard-main\automacao_azure_devops\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{704FCF64-CD8F-4FDD-8446-3A6E09DC6A86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84FA4000-10FD-4EA4-9E0A-DA047F7B8E0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{E79395A8-F579-4870-AAFC-7CF8E73F4ED7}"/>
+    <workbookView xWindow="-18680" yWindow="-250" windowWidth="19180" windowHeight="10060" xr2:uid="{E79395A8-F579-4870-AAFC-7CF8E73F4ED7}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -50,13 +50,13 @@
     <t>Skills</t>
   </si>
   <si>
-    <t>Teste de automação</t>
+    <t>Automação IA</t>
   </si>
   <si>
-    <t>Assigned</t>
+    <t>Open - Scheduling</t>
   </si>
   <si>
-    <t>Automação IA</t>
+    <t>Teste de automação - inicial</t>
   </si>
 </sst>
 </file>
@@ -433,13 +433,45 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="0" row="0">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{5B7B8D5E-0901-4114-8CDF-7671E31E2E5E}">
+  <we:reference id="df76232d-21a6-4463-9d19-0518ac5aab5d" version="1.1.0.0" store="EXCatalog" storeType="EXCatalog"/>
+  <we:alternateReferences>
+    <we:reference id="WA200000556" version="1.1.0.0" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="documentId" value="&quot;50a4d164-ed88-4aad-918b-15571d4dfbf1&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+  <we:extLst>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{D87F86FE-615C-45B5-9D79-34F1136793EB}">
+      <we:containsCustomFunctions/>
+    </a:ext>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{7C84B067-C214-45C3-A712-C9D94CD141B2}">
+      <we:customFunctionIdList>
+        <we:customFunctionIds>_xldudf_JIRA_JQL</we:customFunctionIds>
+      </we:customFunctionIdList>
+    </a:ext>
+  </we:extLst>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CC4A447-7B97-4215-B7D5-CEF450479ABA}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -456,13 +488,13 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Suporta novo layout relacional de vagas
Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/automacao_azure_devops/vagas.xlsx
+++ b/automacao_azure_devops/vagas.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\t.douglas.medeiros\Desktop\dmma-dashboard-main\dmma-dashboard-main\automacao_azure_devops\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://avanade.sharepoint.com/sites/DeliveryOperationsBrazil/Documentos Compartilhados/3 - COE/Esteira de vagas/automacao_azure_devops/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BA51D29-EF6D-4E9A-9F9F-885F19315A35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="50" documentId="13_ncr:1_{3BA51D29-EF6D-4E9A-9F9F-885F19315A35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C8B080A0-B6DE-463F-AD1D-D39051B37E6C}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="380" windowWidth="19180" windowHeight="10060" xr2:uid="{E79395A8-F579-4870-AAFC-7CF8E73F4ED7}"/>
+    <workbookView xWindow="-19310" yWindow="-1720" windowWidth="19420" windowHeight="10300" xr2:uid="{E79395A8-F579-4870-AAFC-7CF8E73F4ED7}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -39,31 +39,189 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>state</t>
-  </si>
-  <si>
-    <t>Skills</t>
-  </si>
-  <si>
-    <t>Automação IA</t>
-  </si>
-  <si>
-    <t>Open - Scheduling</t>
-  </si>
-  <si>
-    <t>Teste de automação - inicial do Tiego´s boy</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="53">
+  <si>
+    <t>Id MyScheduling</t>
+  </si>
+  <si>
+    <t>Status Myscheduling</t>
+  </si>
+  <si>
+    <t>Cliente</t>
+  </si>
+  <si>
+    <t>RoleTitle</t>
+  </si>
+  <si>
+    <t>Skillls</t>
+  </si>
+  <si>
+    <t>Idioma</t>
+  </si>
+  <si>
+    <t>Staffing</t>
+  </si>
+  <si>
+    <t>Role Description</t>
+  </si>
+  <si>
+    <t>Modalidade de Trabalho</t>
+  </si>
+  <si>
+    <t>RolePrimaryContact</t>
+  </si>
+  <si>
+    <t>level_from</t>
+  </si>
+  <si>
+    <t>level_to</t>
+  </si>
+  <si>
+    <t>Prática</t>
+  </si>
+  <si>
+    <t>Sub Prática</t>
+  </si>
+  <si>
+    <t>OppID</t>
+  </si>
+  <si>
+    <t>Account.</t>
+  </si>
+  <si>
+    <t>PROJETO</t>
+  </si>
+  <si>
+    <t>Win Probability</t>
+  </si>
+  <si>
+    <t>Estimated Close Date</t>
+  </si>
+  <si>
+    <t>Status EALA</t>
+  </si>
+  <si>
+    <t>Sales Stage</t>
+  </si>
+  <si>
+    <t>Must Win Deal</t>
+  </si>
+  <si>
+    <t>Forecast category</t>
+  </si>
+  <si>
+    <t>Estimated Project Start Date</t>
+  </si>
+  <si>
+    <t>Estimated Project End Date</t>
+  </si>
+  <si>
+    <t>Channel</t>
+  </si>
+  <si>
+    <t>Role Start Date</t>
+  </si>
+  <si>
+    <t>Role End Date</t>
+  </si>
+  <si>
+    <t>Role Is Overdue</t>
+  </si>
+  <si>
+    <t>DataAberturaScheduling</t>
+  </si>
+  <si>
+    <t>Campos</t>
+  </si>
+  <si>
+    <t>Tipo de Item</t>
+  </si>
+  <si>
+    <t>valor</t>
+  </si>
+  <si>
+    <t>Position</t>
+  </si>
+  <si>
+    <t>Project</t>
+  </si>
+  <si>
+    <t>Open - In Process</t>
+  </si>
+  <si>
+    <t>BANCO BRADESCO</t>
+  </si>
+  <si>
+    <t>[Banco Bradesco] [A000460597] | Dev FullStack  | (PAG) Tribo Recebimento</t>
+  </si>
+  <si>
+    <t>Spring Boot</t>
+  </si>
+  <si>
+    <t>Em branco</t>
+  </si>
+  <si>
+    <t>Andreia Silva Dantas</t>
+  </si>
+  <si>
+    <t>Dev FullStack - Java Springboot + Angular
+Descrição
+Responsabilidades:
+Desenvolver e manter aplicações fullstack utilizando Java (Spring Boot) e Angular
+Construir e integrar APIs RESTful em arquitetura de microserviços
+Garantir qualidade de código, performance e boas práticas de desenvolvimento
+Atuar em conjunto com times ágeis (PO, QA, DevOps)
+Participar de code reviews, troubleshooting e evolução das soluções
+Requisitos:
+Experiência com Java e Spring Boot
+Experiência sólida com Angular (preferencialmente versões recentes)
+Conhecimento em APIs REST, microserviços e integração de sistemas
+Vivência com Git, testes (unitários/TDD) e boas práticas de código
+Conhecimento em SQL e bancos de dados
+Diferenciais:
+Experiência com Cloud (Azure) e práticas de DevOps/CI/CD
+Conhecimento em arquitetura hexagonal ou clean architecture
+Experiência com mensageria, performance e observabilidade</t>
+  </si>
+  <si>
+    <t>Onsite</t>
+  </si>
+  <si>
+    <t>Joao C. Octaviano</t>
+  </si>
+  <si>
+    <t>Applications Practice</t>
+  </si>
+  <si>
+    <t>Software Engineering</t>
+  </si>
+  <si>
+    <t>A000460597</t>
+  </si>
+  <si>
+    <t>BR - Banco Bradesco</t>
+  </si>
+  <si>
+    <t>Projeto sem nome</t>
+  </si>
+  <si>
+    <t>Won</t>
+  </si>
+  <si>
+    <t>5.3 - Realize - Won/Backlog</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Direct</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -72,21 +230,83 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="8"/>
-      <color rgb="FF000000"/>
-      <name val="Segoe UI"/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF92D050"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Aptos"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="0"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor theme="5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -94,13 +314,61 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -116,6 +384,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -467,34 +739,325 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CC4A447-7B97-4215-B7D5-CEF450479ABA}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:AE3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="36" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="62.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.6328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="54.54296875" customWidth="1"/>
+    <col min="10" max="10" width="20.90625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.26953125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.6328125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="22.81640625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="24" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="23.08984375" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="7.54296875" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="13" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="12" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="13.36328125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="20.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="N1" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="O1" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="P1" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q1" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="R1" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="S1" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="T1" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="U1" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="V1" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="W1" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="X1" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y1" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z1" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA1" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="AB1" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="AC1" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="AD1" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="AE1" s="8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C2" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D2" s="10" t="s">
         <v>2</v>
       </c>
+      <c r="E2" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="I2" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="J2" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="K2" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="L2" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="M2" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="N2" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="O2" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="P2" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q2" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="R2" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="S2" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="T2" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="U2" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="V2" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="W2" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="X2" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="Y2" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="Z2" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="AA2" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB2" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="AC2" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="AD2" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="AE2" s="10" t="s">
+        <v>29</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>3</v>
+    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="7">
+        <v>6439485</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="L3" s="4">
+        <v>11</v>
+      </c>
+      <c r="M3" s="4">
+        <v>11</v>
+      </c>
+      <c r="N3" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="O3" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="P3" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q3" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="R3" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="S3" s="4">
+        <v>100</v>
+      </c>
+      <c r="T3" s="6">
+        <v>46132</v>
+      </c>
+      <c r="U3" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="V3" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="W3" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="X3" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="Y3" s="6">
+        <v>46113</v>
+      </c>
+      <c r="Z3" s="6">
+        <v>46448</v>
+      </c>
+      <c r="AA3" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="AB3" s="6">
+        <v>46321</v>
+      </c>
+      <c r="AC3" s="6">
+        <v>46686</v>
+      </c>
+      <c r="AD3" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="AE3" s="6">
+        <v>46237</v>
       </c>
     </row>
   </sheetData>
@@ -502,6 +1065,265 @@
 </worksheet>
 </file>
 
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100834B68D036177D44877082871E69D0CD" ma:contentTypeVersion="12" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="e02c6a46cc97efde99847c4cf4776a40">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="36f4fad3-9057-4459-ba28-7682280a739d" xmlns:ns3="0059ae8e-fd03-4f55-a5d5-28f7b0f0089b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="255b278d5207e6a37bc1262e28a53451" ns2:_="" ns3:_="">
+    <xsd:import namespace="36f4fad3-9057-4459-ba28-7682280a739d"/>
+    <xsd:import namespace="0059ae8e-fd03-4f55-a5d5-28f7b0f0089b"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="36f4fad3-9057-4459-ba28-7682280a739d" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="11" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="12" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="13" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="14" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="15" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="17" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Marcações de imagem" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="1217ff2e-1616-4146-8372-4640400776c3" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="19" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="0059ae8e-fd03-4f55-a5d5-28f7b0f0089b" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="18" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{288a5aaf-9916-4cfe-98c7-000097c39464}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="0059ae8e-fd03-4f55-a5d5-28f7b0f0089b">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de Conteúdo"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="36f4fad3-9057-4459-ba28-7682280a739d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="0059ae8e-fd03-4f55-a5d5-28f7b0f0089b" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9F45952D-E74E-41FA-8139-064CF7A86613}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="36f4fad3-9057-4459-ba28-7682280a739d"/>
+    <ds:schemaRef ds:uri="0059ae8e-fd03-4f55-a5d5-28f7b0f0089b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B69C1ECF-4E4E-4D8C-9323-C2D91D27A047}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="36f4fad3-9057-4459-ba28-7682280a739d"/>
+    <ds:schemaRef ds:uri="0059ae8e-fd03-4f55-a5d5-28f7b0f0089b"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7E1A605A-01BB-4F60-A9F7-B23A1F865D57}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{5fae8262-b78e-4366-8929-a5d6aac95320}" enabled="1" method="Standard" siteId="{cf36141c-ddd7-45a7-b073-111f66d0b30c}" contentBits="0" removed="0"/>

</xml_diff>